<commit_message>
Update Amazon seller master data
</commit_message>
<xml_diff>
--- a/output/Amazon_Seller_Master_Data.xlsx
+++ b/output/Amazon_Seller_Master_Data.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Amazon Sellers" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Amazon Sellers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Amazon Sellers'!$A$1:$U$5</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:U5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -904,8 +904,105 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Men'S Formal Shoes</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr"/>
+      <c r="C5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Cocoblu Retail</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Seller</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Men'S Formal Shoes</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>+919210579250</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>mail@okcalc.com</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>33AAJCC8517E1ZS</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>AAJCC8517E</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr"/>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>Not Found</t>
+        </is>
+      </c>
+      <c r="T5" s="3" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="U5" s="3" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U4"/>
+  <autoFilter ref="A1:U5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>
 </worksheet>

</xml_diff>